<commit_message>
Update test cases with new inputs, expected outputs, and automation results
</commit_message>
<xml_diff>
--- a/IT23740310 - Assignment 1 - Test cases.xlsx
+++ b/IT23740310 - Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omind\Downloads\IT23740310_playwright-main\IT23740310_playwright-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8D59EA-2BFA-4F14-A989-BDB9EE26021E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EEFF954-167F-4443-9DFD-DA073E85D1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="300">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -583,372 +583,364 @@
     <t>Neg_0031</t>
   </si>
   <si>
-    <t>mama 2hrs wtr nidagnna giya</t>
-  </si>
-  <si>
-    <t>මම පැය 2ක් විතර නිදාගන්න ගියා</t>
-  </si>
-  <si>
-    <t>මම දවස් 2ක් විතර නිදාගන්න ගියා</t>
-  </si>
-  <si>
-    <t>Inputs with Numbers and Numeric Suffixes
-Inputs with Time Formats</t>
-  </si>
-  <si>
-    <t>Evidence: “2hrs” includes a number with an English time suffix.
-Rationale: The input refers to a duration/time expression.</t>
+    <t>M</t>
+  </si>
+  <si>
+    <t>oyata dennama wage ahanna one, kohomada oya meka ethakama ignore karanne?</t>
+  </si>
+  <si>
+    <t>ඔයාට දෙන්නම වගේ අහන්න ඕනේ, කොහොමද ඔයා මේකා එතකම ignore කරන්නේ?</t>
+  </si>
+  <si>
+    <t>ඔයාට දෙන්නම වගේ අහන්න ඕනේ, කොහොමද ඔයා මේක එතකම ignore කරන්නේ?</t>
+  </si>
+  <si>
+    <t>Informal Query / Social Interaction</t>
+  </si>
+  <si>
+    <t>Uses colloquial Singlish ('oyata dennama wage ahanna one') to ask a personal question.</t>
   </si>
   <si>
     <t>Neg_0032</t>
   </si>
   <si>
-    <t>api 5pm ta set wenna pulwn</t>
-  </si>
-  <si>
-    <t>අපි 5pm ට සෙට් වෙන්න පුළුවන්</t>
-  </si>
-  <si>
-    <t>අපි 5pm ට set වෙන්න පුළුවන්</t>
-  </si>
-  <si>
-    <t>Inputs with Time Formats</t>
-  </si>
-  <si>
-    <t>Evidence: “5pm” is a time format embedded in the Singlish input.</t>
+    <t>Thatha kiwwa, heta subodha dawasata wakktu walata gedara enname kiyala.</t>
+  </si>
+  <si>
+    <t>තාත්තා කිව්වා, හෙට නියමිත වේලාවට ගෙදර එන්නම කියලා.</t>
+  </si>
+  <si>
+    <t>එන්න කිව්වා, හෙට සුබෝධ දවසට වාක්කුට්ටු වලට ගෙදර එන්නමේ කියලා.</t>
+  </si>
+  <si>
+    <t>Family Communication / Informative</t>
+  </si>
+  <si>
+    <t>Contains family references ('Thatha') and mixed language terms ('wakktu walata').</t>
   </si>
   <si>
     <t>Neg_0033</t>
   </si>
   <si>
-    <t>mta Rs1500k one wnawa</t>
-  </si>
-  <si>
-    <t>මට රුපියල් 1500ක් ඕන වෙලා තියෙනවා</t>
-  </si>
-  <si>
-    <t>මට Rs1500ක් ඕනේ වෙනවා</t>
-  </si>
-  <si>
-    <t>Inputs with Currency</t>
-  </si>
-  <si>
-    <t>Evidence: “Rs1500k” contains a currency marker and numeric amount.</t>
+    <t>Subha Aluth Avuruddak Wewa Dilani akka! Oyata saha pawule semata suba patauma.</t>
+  </si>
+  <si>
+    <t>සුභ අලුත් අවුරුද්දක් වේවා දිලාණි අක්කා! ඔයාට සහ පවුලේ සැමට සුභ ආරම්භයක්.</t>
+  </si>
+  <si>
+    <t>සුභ අලුත් අවුරුද්දක් වේවා දිලානි අක්කා! ඔයාට සහ පවුලේ සැමට සුබ පාටඋම.</t>
+  </si>
+  <si>
+    <t>Greetings / Seasonal</t>
+  </si>
+  <si>
+    <t>Standard festive greeting ('Subha Aluth Avuruddak Wewa') with personal well wishes.</t>
   </si>
   <si>
     <t>Neg_0034</t>
   </si>
   <si>
-    <t>oyta 1st plc eka lbuna neda</t>
-  </si>
-  <si>
-    <t>ඔයාට පළමු ස්ථානය ලැබුණා නේද?</t>
-  </si>
-  <si>
-    <t>ඔයාට 1st plc එක ලැබුණා නේද</t>
-  </si>
-  <si>
-    <t>Inputs with Numbers and Numeric Suffixes</t>
-  </si>
-  <si>
-    <t>Evidence: “1st” is an ordinal numeric suffix in the Singlish input.</t>
+    <t>karunakarala mage laptop eka restart karanna hadala balanna, eka on wenawa ne.</t>
+  </si>
+  <si>
+    <t>කරණාකරලා මගේ laptop එක restart කරන්න හදලා බලන්න, ඒකා on වෙනවා නෑ.</t>
+  </si>
+  <si>
+    <t>කරුණාකරලා මගේ laptop එක restart කරන්න හදලා බලන්න, ඒක ඕං වෙනවා නේ.</t>
+  </si>
+  <si>
+    <t>Technical Support / Request</t>
+  </si>
+  <si>
+    <t>Request for technical help using English terms ('laptop', 'restart') in Singlish syntax.</t>
   </si>
   <si>
     <t>Neg_0035</t>
   </si>
   <si>
-    <t>mama km 2k duwana</t>
-  </si>
-  <si>
-    <t>මම කිලෝමීටර් 2ක් දුවලා</t>
-  </si>
-  <si>
-    <t>මම km 2ක් දුවන</t>
-  </si>
-  <si>
-    <t>Unit of Measurements</t>
-  </si>
-  <si>
-    <t>Evidence: “km 2k” includes the unit “km” and a measurement amount.</t>
+    <t>nah nah, mama meka accept karannam, oyata godak thanks machan.</t>
+  </si>
+  <si>
+    <t>නෑ නෑ, මම මේකා accept කරන්නම්, ඔයාට ගොඩක් thanks මචන්.</t>
+  </si>
+  <si>
+    <t>නාහ් නාහ්, මම මේක accept කරන්නම්, ඔයාට ගොඩක් Thanks මචන්.</t>
+  </si>
+  <si>
+    <t>Expressing Gratitude / Acceptance</t>
+  </si>
+  <si>
+    <t>Casual confirmation and thanks ('accept karannam', 'godak thanks machan').</t>
   </si>
   <si>
     <t>Neg_0036</t>
   </si>
   <si>
-    <t>api sndy dwsata trip ekk ymu</t>
-  </si>
-  <si>
-    <t>අපි සන්ඩේ දවසට ට්‍රිප් එකක් යමු</t>
-  </si>
-  <si>
-    <t>අපි sndy දවසට trip එකක් යමු</t>
-  </si>
-  <si>
-    <t>Dates
-Place Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t>Evidence: “sndy dwsata” refers to a day/date expression.
-Rationale: “trip” context refers to going to a place, but no specific proper place name is included.</t>
+    <t>wada wada kiyanna, nathnam oya kade duwanawa kiyala ape set hemoma dannawa.</t>
+  </si>
+  <si>
+    <t>වඩ වඩ කියන්න, නැත්නම් ඔයා කඩේ දුවනවා කියලා අපේ සෙට් හෙමෝම දන්නවා.</t>
+  </si>
+  <si>
+    <t>වඩා වඩා කියන්න, නැත්නම් ඔය කඩේ දුවනවා කියලා අපේ set හැමෝම දන්නවා.</t>
+  </si>
+  <si>
+    <t>Slang / Group Interaction</t>
+  </si>
+  <si>
+    <t>Uses peer group slang ('ape set hemoma') and informal expressions ('kade duwanawa').</t>
   </si>
   <si>
     <t>Neg_0037</t>
   </si>
   <si>
-    <t>mama nxt wk exam ekk thiyanw</t>
-  </si>
-  <si>
-    <t>මට නෙක්ස්ට් වීක් එක්සෑම් එකක් තියෙනවා</t>
-  </si>
-  <si>
-    <t>මම nxt week exam එකක් තියෙනවා</t>
-  </si>
-  <si>
-    <t>Dates
-English Clipped Forms in Singlish</t>
-  </si>
-  <si>
-    <t>Evidence: “nxt wk” refers to next week.
-Rationale: “nxt” and “wk” are clipped forms of “next” and “week”.</t>
+    <t>mama yanava... oya nadda? nathnam mama ekkai yanne, confirm karanna.</t>
+  </si>
+  <si>
+    <t>මම යනවා... ඔයා නැද්ද? නැත්නම් මම එකාමයි යන්නේ, confirm කරන්න.</t>
+  </si>
+  <si>
+    <t>මම යනවා... ඔයා නැද්ද? නැත්නම් මම එක්කයි යන්නේ, confirm කරන්න.</t>
+  </si>
+  <si>
+    <t>Travel / Coordination</t>
+  </si>
+  <si>
+    <t>Short message for coordination with informal questioning ('oya nadda?', 'confirm karanna').</t>
   </si>
   <si>
     <t>Neg_0038</t>
   </si>
   <si>
-    <t>oyta feb 10 wnda free da</t>
-  </si>
-  <si>
-    <t>ඔයාට පෙබරවාරි 10 වෙනිදා ෆ්‍රී ද?</t>
-  </si>
-  <si>
-    <t>ඔයාට ෆේබර් 10 වෙන්ඩ free ද</t>
-  </si>
-  <si>
-    <t>Inputs with Dates</t>
-  </si>
-  <si>
-    <t>Evidence: “feb 10” is a date expression embedded in the Singlish input.</t>
+    <t>mn oyt adha katha krnnt bae, heta balamu. oya danne da mama busy kiyala?</t>
+  </si>
+  <si>
+    <t>මං ඔයාට අද කතා කරන්න බෑ, හෙට බලමු. ඔයා දන්නේද මම busy කියලා?</t>
+  </si>
+  <si>
+    <t>මන් ඔයාට අද කතා කරන්නත් බැහැ, හෙට බලමු. ඔයා දන්නෑ ද මම busy කියලා?</t>
+  </si>
+  <si>
+    <t>Status Update / Busy</t>
+  </si>
+  <si>
+    <t>Explanation of unavailability using mixed script logic ('mn oyt adha katha krnnt bae').</t>
   </si>
   <si>
     <t>Neg_0039</t>
   </si>
   <si>
-    <t>mtng eka 8.30am ptn gnn</t>
-  </si>
-  <si>
-    <t>මීටින් එක 8.30am පටන් ගන්න</t>
-  </si>
-  <si>
-    <t>මට නම් ඒක 8.30am පටන් ගන්න</t>
-  </si>
-  <si>
-    <t>Evidence: “8.30am” is a time format embedded in the Singlish input.</t>
+    <t>api ada lunch ganna Burger King ekata yamuda? mama office eken 1 walata free.</t>
+  </si>
+  <si>
+    <t>අපි අද lunch ගන්න Burger King එකාට යමුද? මම office ඒකෙං 1 වලට free.</t>
+  </si>
+  <si>
+    <t>අපි අද lunch ගන්න Burger King එකට යමුද? මම office එකෙන් 1 වලට free.</t>
+  </si>
+  <si>
+    <t>Social Planning / Food</t>
+  </si>
+  <si>
+    <t>Casual suggestion for lunch at a specific brand ('Burger King') with time reference.</t>
   </si>
   <si>
     <t>Neg_0040</t>
   </si>
   <si>
-    <t>api dec wlata plan ekk hdmu</t>
-  </si>
-  <si>
-    <t>අපි දෙසැම්බර් වලට ප්ලෑන් එකක් හදමු</t>
-  </si>
-  <si>
-    <t>අපි දෙසැම්බර් වලට plan එකක් හදමු</t>
-  </si>
-  <si>
-    <t>Evidence: “dec” refers to December, a month/date expression.</t>
+    <t>mama already on the way, traffic nisa poddak late wenawa. sorry bro.</t>
+  </si>
+  <si>
+    <t>මම already on the way, traffic නිසා පොඩ්ඩක් late වෙනවා. sorry bro.</t>
+  </si>
+  <si>
+    <t>Travel Status / Apology</t>
+  </si>
+  <si>
+    <t>Informs about traffic and delay ('on the way', 'traffic nisa') with an apology.</t>
   </si>
   <si>
     <t>Neg_0041</t>
   </si>
   <si>
-    <t>ane mchn uba mara hondi</t>
-  </si>
-  <si>
-    <t>අනේ මචං, උඹ මාර හොඳයි</t>
-  </si>
-  <si>
-    <t>අනේ මචන් උඹ මාර හොඳයි</t>
-  </si>
-  <si>
-    <t>Slang and Casual Phrasing
-Greetings</t>
-  </si>
-  <si>
-    <t>Evidence: “mchn” is a casual address/opening.
-Rationale: The sentence uses informal slang such as “uba” and “mara”.</t>
+    <t>oyalage gedara Bluetooth speaker eka charge wenawada? battery dead wage.</t>
+  </si>
+  <si>
+    <t>ඔයාලගේ ගෙදර Bluetooth speaker එකා charge වෙනවාද? battery dead වගේ.</t>
+  </si>
+  <si>
+    <t>ඔයාලගේ ගෙදර Bluetooth speaker එක charge වෙනවද? battery dead වගේ.</t>
+  </si>
+  <si>
+    <t>Household Request / Hardware</t>
+  </si>
+  <si>
+    <t>Inquiry about electronic device ('Bluetooth speaker') and battery status.</t>
   </si>
   <si>
     <t>Neg_0042</t>
   </si>
   <si>
-    <t>sirwt@# meka supiri wdk!!</t>
-  </si>
-  <si>
-    <t>සිරාවට මේක සුපිරි වැඩක්</t>
-  </si>
-  <si>
-    <t>සිරාවට මේක සුපිරි වැඩක්!!</t>
-  </si>
-  <si>
-    <t>Slang and Casual Phrasing</t>
-  </si>
-  <si>
-    <t>Evidence: “sirwt” and “supiri” are casual/slang Singlish expressions.</t>
+    <t>ape class eka Teams eken da nadda? teacher kiwwa link eka Slack eken ewanna.</t>
+  </si>
+  <si>
+    <t>අපේ class එකා Teams ඒකෙං ද නැද්ද? teacher කිව්වා link එකා Slack ඒකෙං එවන්න.</t>
+  </si>
+  <si>
+    <t>අපේ class එක Teams එකෙන් ද නැද්ද? teacher කිව්වා link එක Slack එකෙන් එවන්න.</t>
+  </si>
+  <si>
+    <t>Education / Online Tools</t>
+  </si>
+  <si>
+    <t>Context of online classes using platform names ('Teams', 'Slack').</t>
   </si>
   <si>
     <t>Neg_0043</t>
   </si>
   <si>
-    <t>oy##ta mnwda krnne!!</t>
-  </si>
-  <si>
-    <t>ඔයාට මොනවාද කරන්නේ?</t>
-  </si>
-  <si>
-    <t>ඔයාට මොනවාද කරන්නේ!!</t>
-  </si>
-  <si>
-    <t>Evidence: “ubta” and “bri wei” are informal casual phrasing.</t>
+    <t>Project eka ASAP submit karanna kiwwa, but deadline eka extend una kiyala HR kiwwa.</t>
+  </si>
+  <si>
+    <t>Project එකා ASAP submit කරන්න කිව්වා, but deadline එකා extend උනා කියලා HR කිව්වා.</t>
+  </si>
+  <si>
+    <t>ප්රොජෙක්ට් එක ASAP submit කරන්න කිව්වා, but deadline එක extend වුණා කියලා HR කිව්වා.</t>
+  </si>
+  <si>
+    <t>Work / Corporate Communication</t>
+  </si>
+  <si>
+    <t>Business context regarding deadlines and HR notifications ('ASAP submit', 'HR kiwwa').</t>
   </si>
   <si>
     <t>Neg_0044</t>
   </si>
   <si>
-    <t>mage yluwo set ek dn inne</t>
-  </si>
-  <si>
-    <t>මගේ යාලුවෝ සෙට් එක දැන් කැෆේ එකේ ඉන්නේ</t>
-  </si>
-  <si>
-    <t>මගේ යාළුවෝ set එක දැන් ඉන්නේ</t>
-  </si>
-  <si>
-    <t>Slang and Casual Phrasing
-Place Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t>Rationale: “yluwo set ek” is casual phrasing.
-Evidence: Expected output mentions “කැෆේ එකේ”, indicating a place/location embedded in the sentence.</t>
+    <t>ape gym session eka cancel una, coach naha nisa. next week Monday karamu.</t>
+  </si>
+  <si>
+    <t>අපේ gym session එකා cancel උනා, coach නෑ නිසා. next week Monday කරමු.</t>
+  </si>
+  <si>
+    <t>අපේ gym session එක cancel වුණා, coach නැහැ නිසා. next week Monday කරමු.</t>
+  </si>
+  <si>
+    <t>Health &amp; Fitness / Scheduling</t>
+  </si>
+  <si>
+    <t>Cancelling a session ('gym session', 'cancel una') and rescheduling.</t>
   </si>
   <si>
     <t>Neg_0045</t>
   </si>
   <si>
-    <t>cafe ek</t>
-  </si>
-  <si>
-    <t>කැෆේ එක</t>
-  </si>
-  <si>
-    <t>cafe එක</t>
-  </si>
-  <si>
-    <t>Place Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t>Evidence: “cafe” is used as a location/place term in the input.</t>
+    <t>mama adiya 15k witharai giya heta, eka km ekkai balagena enna one thamai.</t>
+  </si>
+  <si>
+    <t>මම අඩිය 15k විතරයි ගියා, ඒකා km එකක් බලාගෙන එන්න ඕනේ තමයි.</t>
+  </si>
+  <si>
+    <t>මම අඩිය 15ක් විතරයි ගියා හෙට, එක කිම් එක්කයි බලාගෙන එන්න ඕනේ තමයි.</t>
+  </si>
+  <si>
+    <t>Travel / Distance</t>
+  </si>
+  <si>
+    <t>Mixed measurement and plan description ('adiya 15k', 'km ekkai').</t>
   </si>
   <si>
     <t>Neg_0046</t>
   </si>
   <si>
-    <t>mama dn tika upset wela inne</t>
-  </si>
-  <si>
-    <t>මම දැන් ටිකක් අප්සෙට් වෙලා ඉන්නේ</t>
-  </si>
-  <si>
-    <t>මම දැන් ටික upset වෙලා ඉන්නේ</t>
-  </si>
-  <si>
-    <t>Responses
-English Clipped Forms in Singlish</t>
-  </si>
-  <si>
-    <t>Rationale: The input is a status/response about feeling upset.
-Evidence: “dn” is a clipped form of “dan”/now.</t>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Machan, mama oyata godak kalin kiwwa meka plan karanna kiyala. Ada hawasa 6:30PM walata Zoom call ekai thiyenne, oya office eken pitath wenna agena join karanna. Karunakarala network connection eka sari karala headphones dala camera on karala ready wenna. Mage WhatsApp eke message eka diha balagena confirm karanna. Nathnam @Sachith ayye kiyana kiyala kiyamu. Thanks bro elakiri da meka!</t>
+  </si>
+  <si>
+    <t>මචන්, මම ඔයාට ගොඩක් කලින් කිව්වා මේකා plan කරන්න කියලා. අද හවස 6:30PM වලට Zoom call එකක් තියෙනවා, ඔයා office ඒකෙං පිටත් වෙන්නාගෙන join කරන්න. කරුණාකරලා network connection එකා සරි කරලා headphones දාලා camera on කරලා ready වෙන්න. මගේ WhatsApp ඒකේ message එකා දිහා බලාගෙන confirm කරන්න. නැත්නම් @Sachith අය්යා කියනවා කියලා කියමු. Thanks bro elakiri ද මේකා!</t>
+  </si>
+  <si>
+    <t>මචන්, මම ඔයාට ගොඩක් කලින් කිව්වා මේක ප්ලෑන් කරන්න කියලා. අද හවස 6:30PM වලට Zoom call එකයි තියෙන්නේ, ඔයා office එකෙන් පිටත් වෙන්න ආගෙන join කරන්න. කරුණාකරලා network connection එක සාරි කරලා headphones දාලා camera on කරලා ready වෙන්න. මගේ WhatsApp එකේ message එක දිහා බලාගෙන confirm කරන්න. නැත්නම් @සචිත් අය්යේ කියන කියලා කියමු. Thanks bro එළකිරි ද මේක!</t>
+  </si>
+  <si>
+    <t>Complex Coordination / Technical Instructions</t>
+  </si>
+  <si>
+    <t>Long paragraph involving time, Zoom links, hardware setup, and tag references (@Sachith).</t>
   </si>
   <si>
     <t>Neg_0047</t>
   </si>
   <si>
-    <t>me link ek open krla blnna https//abcccom</t>
-  </si>
-  <si>
-    <t>මේ ලින්ක් එක ඔපන් කරලා බලන්න https://abc.com</t>
+    <t>Akka, mama meka oyata explain karanna hadanawa. Api heta 2026-05-12 ta school trip eka Nuwara Eliya walata yamu kiyala plan karala thiyenawa. Bus eka subodha dawasa 7:00AM ta school eke inna pitath wenawa. Lamayinta Rs.1500 ganna one, lunch school kadeta dila tiyenawa. Priyantha ayya kiwwa heta confirm karanna one kiyala. Please ASAP meka confirm karala mama hata WhatsApp eke message ekak ewanna.</t>
+  </si>
+  <si>
+    <t>අක්කා, මම මේකා ඔයාට explain කරන්න හදනවා. අපි හෙට 2026-05-12 ට school trip එකා Nuwara Eliya වලට යමු කියලා plan කරලා තිියයි. Bus එකා 7:00AM ට school ඒකෙං පිටත් වෙනවා. ළමයින්ට Rs.1500 ගන්න ඕනේ, lunch school කඩේට දීලා තිියයි. Priyantha අය්යා කිව්වා හෙට confirm කරන්න ඕනේ කියලා. Please ASAP මේකා confirm කරලා මම හට WhatsApp ඒකේ message එකක් එවන්න.</t>
   </si>
   <si>
     <t>මේ link එක open කරලා බලන්න https//abcccom</t>
   </si>
   <si>
-    <t>Online Identifiers in Singlish
-Inputs with Punctuation Marks</t>
-  </si>
-  <si>
-    <t>Evidence: The input contains a URL-like online identifier “https//abcccom”.
-Rationale: The expected output normalizes it with punctuation as “https://abc.com”.</t>
+    <t>Event Planning / Detailed Travel</t>
+  </si>
+  <si>
+    <t>Detailed itinerary for a school trip with dates, costs, and specific instructions.</t>
   </si>
   <si>
     <t>Neg_0048</t>
   </si>
   <si>
-    <t>oyta email ekk ewnna pulwnd</t>
-  </si>
-  <si>
-    <t>ඔයාට ඊමේල් එකක් එවන්න පුළුවන්ද?</t>
-  </si>
-  <si>
-    <t>ඔයාට email එකක් එවන්න පුළුවන්ද</t>
-  </si>
-  <si>
-    <t>Online Identifiers in Singlish
-Question forms</t>
-  </si>
-  <si>
-    <t>Evidence: “email” is an online communication identifier/term.
-Rationale: “pulwnd” asks whether it is possible.</t>
+    <t>Machan 😂 oya dannawada ada match eka kohoma una kiyala? Kavindu aiye 💪 mara batting karapu, 120 run dala team geluwa. Uba nethuwa eka ballath game eke naha 😅. Mama Rs.500 bet eka dunna machan Tharindu aiyata, dan uba Rs.500 denna one. Heta office eka 9:00AM ta early enna one, boss kiwwa ASAP update eka ewanna kiyala. Oya enna nam dennama yamu 🙂 api late wunoth boss angry wenawa ne 😬</t>
+  </si>
+  <si>
+    <t>මචන් 😂 ඔයා දන්නවාද අද match එකා කොහොම උනා කියලා? කවිඳු අය්යා 💪 මාර batting කාරාපු, 120 run දාලා team ගෙලුවා. උඹ නෙතුවා ඒකා ballath game ඒකේ නෑ 😅. මම Rs.500 bet එකා දුන්නා මචන් තාරිඳු අය්යාට, දන් උඹ Rs.500 දෙන්න ඕනේ. හෙට office ඒකා 9:00AM ට early එන්න ඕනේ, boss කිව්වා ASAP update එකා එවන්න කියලා. ඔයා එනනම් දෙන්නමයි යමු 🙂 අපි late උනොත් boss angry වෙනවා නේ 😬</t>
+  </si>
+  <si>
+    <t>අක්කා, මම මේක ඔයාට explain කරන්න හදනවා. අපි හෙට 2026-05-12 ට school trip එක නුවර එළිය වලට යමු කියලා plan කරලා තියෙනවා. බස් එක සුබෝද දවස 7:00AM ට school එකේ ඉන්න පිටත් වෙනවා. ළමයින්ට Rs.1500 ගන්න ඕනේ, lunch school කඩේට දිලා තියෙනවා. ප්රියන්ත අයියා කිව්වා හෙට confirm කරන්න ඕනේ කියලා. Please ASAP මේක confirm කරලා මම හට WhatsApp ඒකේ message එකක් එවන්න.</t>
+  </si>
+  <si>
+    <t>Sports / Financial / Social</t>
+  </si>
+  <si>
+    <t>High-length input with emotional markers (emojis), match results, bet info, and work warnings.</t>
   </si>
   <si>
     <t>Neg_0049</t>
   </si>
   <si>
-    <t>mta whatsapp msg ekk dnn</t>
-  </si>
-  <si>
-    <t>මට වට්ස්ඇප් මැසේජ් එකක් දාන්න</t>
-  </si>
-  <si>
-    <t>මට whatsapp msg එකක් දාන්න</t>
-  </si>
-  <si>
-    <t>Platform/App Names in Singlish
-Command forms</t>
-  </si>
-  <si>
-    <t>Evidence: “whatsapp” is an app/platform name.
-Rationale: “dnn” functions as a command to send/post the message.</t>
+    <t>Bro elakiri, mama oyata kiyannam meka sheer hard work. Mama kilomitara 10k witharai ran. Subodha dawasa 6:00AM ta start karala ran, 42 minutes witharai giyaa. Oyath try karanna hadanna, nathnam mama oyata Strava eke link eka share karannam. Api dennama heta payin yamu, www.mapmyrun.com eke route eka balala plan karamu. Oyage email eka ewanna: bro123@gmail.com. Mama ASAP reply karannam.</t>
+  </si>
+  <si>
+    <t>Bro elakiri, මම ඔයාට කියන්නම් මේකා sheer hard work. මම කිලෝමීටර 10k විතර දිව්වා. සුබොධ දවස 6:00AM ට start කරලා දිව්වා, 42 minutes විතරයි ගියා. ඔයාත් try කරන්න හදන්නා, නැත්නම් මම ඔයාට Strava ඒකේ link එකා share කරන්නම්. අපි දෙන්නම හෙට පයින් යමු, www.mapmyrun.com ඒකේ route එකා බලලා plan කරමු. ඔයාගේ email එකාට එවන්නා: bro123@gmail.com. මම ASAP reply කරන්නම්.</t>
+  </si>
+  <si>
+    <t>මචං 😂 ඔයා දන්නවද අද match එක කොහොම වුණා කියලා? කවිඳු අයියෙ 🤣 මාර batting කරපු, 120 රූන් දාලා team ගැලුවා. උඹ නැතුව ඒක බල්ලත් ගමේ එකේ නැහැ 😅. මම Rs.500 බැට් එක දුන්නා මචං තරිඳු අයියාට, දැන් උඹ Rs.500 දෙන්න ඕනේ. හෙට office එක 9:00AM ට early එන්න ඕනේ, boss කිව්වා ASAP update එක එවන්න කියලා. ඔයා එන්න නම් දෙන්නම යමු 🙂 අපි late වුණොත් boss angry වෙනවා නේ</t>
+  </si>
+  <si>
+    <t>Health &amp; Fitness / Digital Integration</t>
+  </si>
+  <si>
+    <t>Detailed description of a run with specific stats, Strava links, and website references.</t>
   </si>
   <si>
     <t>Neg_0050</t>
   </si>
   <si>
-    <t>@kasun oyta meka blnna pulwnd</t>
-  </si>
-  <si>
-    <t>@කසුන් ඔයාට මේක බලන්න පුළුවන්ද?</t>
-  </si>
-  <si>
-    <t>@කසුන් ඔයාට මේක බලන්න පුළුවන්ද</t>
-  </si>
-  <si>
-    <t>Online Identifiers in Singlish
-Person Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t>Evidence: “@kasun” is an online mention/identifier.
-Rationale: “kasun” is a person name embedded in the Singlish input.</t>
+    <t>Ane machan, oya dannawada ada kohomada una kiyala? Subodha dawasa nisa office band una. Mama geyata awa bus eken, Rs.350 ticket eka gatta. Gedara awa balana kotath WiFi naha, SLT kattiya weda karana kiyala. Mama meka ASAP fix karanna kiyanneth bahayi. Heta 8:00AM ta technician kenekuth enawa kiwwa. Oyath gedara innawada heta? Api dennama inna nam mama oyta 2026-05-10 ta kollo balamu.</t>
+  </si>
+  <si>
+    <t>අනේ මචන්, ඔයා දන්නවාද අද කොහොම උනා කියලා? සුබොධ දවස නිසා office band උනා. මම ගෙදරට ආවා bus ඒකෙං, Rs.350 ticket එකා ගත්තා. ගෙදර ආවා බලනකොතත් WiFi නෑ, SLT කට්ටිය වැඩ කරනවා කියලා. මම මේකා ASAP fix කරන්නා කියන්නත් බෑ. හෙට 8:00AM ට technician කෙනෙකුත් එනවා කිව්වා. ඔයාත් ගෙදර ඉන්නවාද හෙට? අපි දෙන්නම ඉන්නනම් මම ඔයාට 2026-05-10 ට කොල්ලො බලමු.</t>
+  </si>
+  <si>
+    <t>bro එළකිරි, මම ඔයාට කියන්නම් මේක ශීර් හර්ඩ් වොක්. මම කිලෝමිටර 10ක් විතරයි රන්. සුබදහ දවස 6:00AM ට start කරලා රන්, 42 minutes විතරයි ගියා. ඔයත් try කරන්න හදන්න, නැත්නම් මම ඔයාට ස්ට්රාව එකේ link එක share කරන්නම්. අපි දෙන්නම හෙට පයින් යමු, www.mapmyrun.කොම් එකේ route එක බලලා plan කරමු. ඔයාගේ email එක එවන්න: bro123@gmail.කොම්. මම ASAP reply කරන්නම්.</t>
+  </si>
+  <si>
+    <t>Service Disruption / Travel</t>
+  </si>
+  <si>
+    <t>Long explanation of an office closure, travel costs, and WiFi technical issues.</t>
   </si>
 </sst>
 </file>
@@ -3099,25 +3091,25 @@
         <v>179</v>
       </c>
       <c r="B122" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D122" s="11" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E122" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F122" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3152,28 +3144,28 @@
     </row>
     <row r="126" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B126" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D126" s="11" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E126" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F126" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3208,28 +3200,28 @@
     </row>
     <row r="130" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B130" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D130" s="11" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E130" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F130" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H130" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3264,28 +3256,28 @@
     </row>
     <row r="134" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="10" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B134" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D134" s="11" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E134" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F134" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3320,28 +3312,28 @@
     </row>
     <row r="138" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B138" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D138" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E138" s="11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F138" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3376,28 +3368,28 @@
     </row>
     <row r="142" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="10" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B142" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D142" s="11" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E142" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F142" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G142" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3432,28 +3424,28 @@
     </row>
     <row r="146" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B146" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D146" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E146" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F146" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3488,28 +3480,28 @@
     </row>
     <row r="150" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B150" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D150" s="11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E150" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F150" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G150" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3544,28 +3536,28 @@
     </row>
     <row r="154" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B154" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D154" s="11" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E154" s="11" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F154" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G154" s="3" t="s">
-        <v>189</v>
+        <v>232</v>
       </c>
       <c r="H154" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3600,28 +3592,28 @@
     </row>
     <row r="158" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B158" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D158" s="11" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E158" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F158" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G158" s="3" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="H158" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3656,28 +3648,28 @@
     </row>
     <row r="162" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="10" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B162" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D162" s="11" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E162" s="11" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F162" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G162" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="H162" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3712,28 +3704,28 @@
     </row>
     <row r="166" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="10" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B166" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D166" s="11" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E166" s="9" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F166" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G166" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3768,28 +3760,28 @@
     </row>
     <row r="170" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B170" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D170" s="11" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E170" s="11" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F170" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G170" s="3" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="H170" s="3" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3824,28 +3816,28 @@
     </row>
     <row r="174" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="10" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B174" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="D174" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E174" s="9" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F174" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G174" s="3" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="H174" s="3" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3880,28 +3872,28 @@
     </row>
     <row r="178" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="10" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B178" s="8" t="s">
-        <v>9</v>
+        <v>180</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D178" s="11" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E178" s="11" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F178" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G178" s="3" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="H178" s="3" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
     </row>
     <row r="179" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3936,28 +3928,28 @@
     </row>
     <row r="182" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B182" s="8" t="s">
-        <v>9</v>
+        <v>270</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D182" s="11" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="E182" s="9" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="F182" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G182" s="3" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="H182" s="3" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="183" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3992,28 +3984,28 @@
     </row>
     <row r="186" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="10" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B186" s="8" t="s">
-        <v>9</v>
+        <v>270</v>
       </c>
       <c r="C186" s="5" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D186" s="11" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="E186" s="11" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="F186" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G186" s="3" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H186" s="3" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
     </row>
     <row r="187" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4048,28 +4040,28 @@
     </row>
     <row r="190" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="10" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B190" s="8" t="s">
-        <v>9</v>
+        <v>270</v>
       </c>
       <c r="C190" s="5" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="D190" s="11" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="E190" s="9" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="F190" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G190" s="3" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="H190" s="3" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4104,28 +4096,28 @@
     </row>
     <row r="194" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="10" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="B194" s="8" t="s">
-        <v>9</v>
+        <v>270</v>
       </c>
       <c r="C194" s="5" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="D194" s="11" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="E194" s="11" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="F194" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G194" s="3" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="H194" s="3" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4160,28 +4152,28 @@
     </row>
     <row r="198" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="10" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B198" s="8" t="s">
-        <v>9</v>
+        <v>270</v>
       </c>
       <c r="C198" s="5" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="D198" s="11" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E198" s="9" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="F198" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G198" s="3" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="H198" s="3" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4477,9 +4469,9 @@
     <mergeCell ref="E158:E161"/>
     <mergeCell ref="B166:B169"/>
     <mergeCell ref="B118:B121"/>
+    <mergeCell ref="E154:E157"/>
     <mergeCell ref="F94:F97"/>
     <mergeCell ref="E110:E113"/>
-    <mergeCell ref="E154:E157"/>
     <mergeCell ref="F98:F101"/>
     <mergeCell ref="F30:F33"/>
     <mergeCell ref="A30:A33"/>
@@ -4506,8 +4498,8 @@
     <mergeCell ref="A66:A69"/>
     <mergeCell ref="A118:A121"/>
     <mergeCell ref="C14:C17"/>
+    <mergeCell ref="C98:C101"/>
     <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C98:C101"/>
     <mergeCell ref="C154:C157"/>
     <mergeCell ref="E14:E17"/>
     <mergeCell ref="A166:A169"/>

</xml_diff>